<commit_message>
DRAFT v3: update /sdi for two Thursdays, The Mountaineers and the new cost display
Draft only, on a preview branch. Not merged to main, so /sdi on the production
domain is unchanged until Brad approves.

Replaces every hosted file with SDI-Launch-Package-2026-10-06-v3-DRAFT, rebuilds the
complete-package zip, and regenerates all thumbnails and previews.

Page copy follows the v3 brief: both Thursdays (Nov 5 and Nov 12), The Mountaineers
Boardroom venue, the cost pair with "A $497 value" beneath it plus the six-item value
list, "Credentialed Guides that Share the Journey" with the single-guide wording, a
six-week timeline, "create the two Events", and the new registration note. Removes the
free/donation, Central Co-op and take-home wording. Date label is October 6, 2026.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/sdi/SDI_Outreach_Workbook.xlsx
+++ b/public/downloads/sdi/SDI_Outreach_Workbook.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Visit Plan'!$A$1:$R$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Social Groups'!$A$1:$M$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Event Listings'!$A$1:$M$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Launch Calendar'!$A$1:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Launch Calendar'!$A$1:$D$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -566,28 +566,28 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Thursday, Nov 5, 2026, 6:30 to 8:30 PM. Central Co-op, 4502 N Pearl St, Tacoma, WA 98407.</t>
+          <t>Two Thursdays to choose from: Nov 5 or Nov 12, 2026, 6:30 to 8:30 PM on both. The Mountaineers (Boardroom), 2302 N 30th St, Tacoma, WA 98403.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Free launch. A $497 value.</t>
+          <t>Cost: $35 early bird through Oct 29, $50 advance, $60 at the door.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Suggested donation: $35 early bird through Oct 29, $50 advance, $60 at the door.</t>
+          <t>A $497 value. Includes: two hours led by a credentialed guide who walks this road alongside you; a daily writing practice adapted from The Artist's Way by Julia Cameron; growing awareness of the experience of heart, mind, and body alignment; ways to name what you feel, even when words won't come; gentle movement; a clear structure for practice.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Register: soaringdragonflyinstitute.com. Guides: Credentialed Guides with Lived Experience. Use the exact Notice and Disclaimer on anything that describes the session. Avoid: therapy, therapeutic, treatment, clinical, healing, heal, client. Say participant and closing practice. Never mention Medicaid or insurance. Not sponsored by Central Co-op.</t>
+          <t>Register: soaringdragonflyinstitute.com. Guides: Credentialed Guides that Share the Journey. One of the three named guides leads each evening; when naming all three, add: One of these credentialed guides will lead your evening. Use the exact Notice and Disclaimer on anything that describes the session. Avoid: therapy, therapeutic, treatment, clinical, healing, heal, client. Say participant and closing practice. Never mention Medicaid or insurance.</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Event Listings: free calendars and submission pages, with a suggested submit-by date.</t>
+          <t>Event Listings: calendars and submission pages, with a suggested submit-by date.</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Launch Calendar: week-by-week checklist from Oct 5 to Nov 6 with an owner for each task.</t>
+          <t>Launch Calendar: week-by-week checklist from Oct 5 to Nov 13 with an owner for each task.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>6. Center for Spiritual Living holds a Thursday 7 PM meditation that overlaps Nov 5. Ask before assuming they will help.</t>
+          <t>6. Center for Spiritual Living holds a Thursday 7 PM meditation that overlaps both Thursdays (Nov 5 and Nov 12). Ask before assuming they will help.</t>
         </is>
       </c>
     </row>
@@ -692,6 +692,13 @@
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>7. Several listing sites had no fee or deadline information available. Treat "not found" as "ask or check the form".</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>8. Walking clusters and priorities were set around the earlier venue address. The new venue is 2302 N 30th St, so review the Priority A choices against distance before you walk.</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1036,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>Ask before class rush; pitch as free community event, offer a rack card for the front desk.</t>
+          <t>Ask before class rush; pitch as a community evening, offer a rack card for the front desk.</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -1114,7 +1121,7 @@
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>Runs Artist's Way groups and Thursday meditation, nearly identical audience. Note the Nov 5 event is also a Thursday evening; check overlap.</t>
+          <t>Runs Artist's Way groups and Thursday meditation, nearly identical audience. Note the events are on Thursday evenings (Nov 5 and Nov 12); check overlap.</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -1349,12 +1356,12 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Highest proximity; tell them the event is on their block.</t>
+          <t>Neighborhood business; ask if they will display a poster.</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
         <is>
-          <t>Next door to the venue address (4502 N Pearl); neighbors may attend and can walk over.</t>
+          <t>Neighborhood audience; owner may be glad to display a poster.</t>
         </is>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1429,7 +1436,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>Ask owner about cross-promotion; very close to venue.</t>
+          <t>Ask owner about cross-promotion.</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1509,12 +1516,12 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>Closest cluster to venue; walk in between class blocks.</t>
+          <t>Walk in between class blocks.</t>
         </is>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
-          <t>Walkable from the event venue; joint-friendly small-group clients.</t>
+          <t>Joint-friendly small-group clients.</t>
         </is>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -1674,7 +1681,7 @@
       </c>
       <c r="K12" s="7" t="inlineStr">
         <is>
-          <t>Closest library to venue; community board commonly used.</t>
+          <t>Community board commonly used.</t>
         </is>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -1754,7 +1761,7 @@
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Group practice a block from the venue area; therapists can refer clients to a non-clinical circle.</t>
+          <t>Group practice; therapists can refer clients to a non-clinical circle.</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -4314,7 +4321,7 @@
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>Natural foods shopper audience; farther from venue.</t>
+          <t>Natural foods shopper audience; outlying location.</t>
         </is>
       </c>
       <c r="L45" s="7" t="inlineStr">
@@ -5888,7 +5895,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Message admin first; frame as free community resource</t>
+          <t>Message admin first; frame as a community resource</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
@@ -6517,7 +6524,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Meditation and Buddhist teachings, weekly Wednesday sessions, donation based</t>
+          <t>Meditation and Buddhist teachings, weekly Wednesday sessions</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -6886,7 +6893,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Nextdoor policy: businesses must use free Business Pages; neighbors may post nonprofit/community posts up to once weekly (per Nextdoor blog); groups have admin rules</t>
+          <t>Nextdoor policy: businesses must use Business Pages (no fee); neighbors may post nonprofit/community posts up to once weekly (per Nextdoor blog); groups have admin rules</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
@@ -6930,7 +6937,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Free weekly email, Thursdays; events and things to do section</t>
+          <t>Weekly email, Thursdays; events and things to do section</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -6945,7 +6952,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Advertising program offered; no free submission method found</t>
+          <t>Advertising program offered; only a paid advertising option found</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -7638,7 +7645,7 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Eckankar sponsored spirituality conversations, free</t>
+          <t>Eckankar sponsored spirituality conversations</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -7874,7 +7881,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Free online meditation and mindfulness, Seattle based</t>
+          <t>Online meditation and mindfulness, Seattle based</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -8468,7 +8475,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Image 300x300 min, 2000x2000 max; paste plain text; use Custom pricing for free/donation</t>
+          <t>Image 300x300 min, 2000x2000 max; paste plain text; use ticket price tiers for the early bird, advance and door prices</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
@@ -8512,7 +8519,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Posting free; promotion paid. Sources conflict: $20 per location (7 days) vs $2 per community per day (support article)</t>
+          <t>No fee to post; promotion paid. Sources conflict: $20 per location (7 days) vs $2 per community per day (support article)</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -8527,7 +8534,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Local account verification; image 1200x900; title, free/paid, location, description</t>
+          <t>Local account verification; image 1200x900; title, price, location, description</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -8630,7 +8637,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Free; donation encouraged</t>
+          <t>No fee</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -8689,7 +8696,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>No fee</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -8748,7 +8755,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>not stated (appears free)</t>
+          <t>not stated (appears no fee)</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -8925,7 +8932,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Free events: unlimited at no cost; paid tickets 3.7% + $1.79 per ticket + 2.9% processing</t>
+          <t>Events without ticket fees: unlimited at no cost; paid tickets 3.7% + $1.79 per ticket + 2.9% processing</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -8940,12 +8947,12 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Account required; donations would need ticketing setup (not verified)</t>
+          <t>Account required; ticketing setup needed for paid tickets (not verified)</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Registration helps headcount; free event fees nil</t>
+          <t>Registration helps headcount; fees for paid tickets not verified</t>
         </is>
       </c>
       <c r="J10" s="7" t="inlineStr">
@@ -9043,7 +9050,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Appears free (not stated)</t>
+          <t>Appears no fee (not stated)</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -9810,7 +9817,7 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Free for Business Page posts; ads optional paid</t>
+          <t>No fee for Business Page posts; ads optional paid</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -10063,7 +10070,7 @@
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>2. Message the admin before posting, especially in groups that require approval for any promotional post. A short note (what, when, where, free, non-clinical) beats a surprise post that gets deleted.</t>
+          <t>2. Message the admin before posting, especially in groups that require approval for any promotional post. A short note (what, when, where, cost, non-clinical) beats a surprise post that gets deleted.</t>
         </is>
       </c>
     </row>
@@ -10091,7 +10098,7 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>6. Lead with what attendees get and say plainly "free launch, suggested donation, non-clinical." Avoid therapy, healing or treatment claims; some groups (recovery, mental health) restrict anything that sounds like clinical services, and the event is not a substitute for therapy.</t>
+          <t>6. Lead with what attendees get and say plainly the dates, the cost and "non-clinical." Avoid therapy, healing or treatment claims; some groups (recovery, mental health) restrict anything that sounds like clinical services, and the event is not a substitute for therapy.</t>
         </is>
       </c>
     </row>
@@ -10105,7 +10112,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>8. On Nextdoor, posts go to specific neighborhoods, so each area needs its own post. Nextdoor's published policy says businesses should use free Business Pages rather than personal accounts, and that nonprofit and community posts are limited to about once a week for neighbors (https://blog.nextdoor.com/self-promotion-update). Flagged posts stay visible but reach fewer people.</t>
+          <t>8. On Nextdoor, posts go to specific neighborhoods, so each area needs its own post. Nextdoor's published policy says businesses should use Business Pages (no fee) rather than personal accounts, and that nonprofit and community posts are limited to about once a week for neighbors (https://blog.nextdoor.com/self-promotion-update). Flagged posts stay visible but reach fewer people.</t>
         </is>
       </c>
     </row>
@@ -10141,7 +10148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10221,7 +10228,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Create the Facebook Event using the event cover and description in the Directional Document. Invite page followers.</t>
+          <t>Create two Facebook Events (Nov 5 and Nov 12) using the event cover and the description in the playbook. Invite page followers.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr"/>
@@ -10257,7 +10264,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Submit free listings marked Oct 5 or Oct 6 on the Event Listings tab (Eventbrite, Visit Tacoma-Pierce County, Tacoma Weekly, News Tribune).</t>
+          <t>Submit listings marked Oct 5 or Oct 6 on the Event Listings tab (Eventbrite, Visit Tacoma-Pierce County, Tacoma Weekly, News Tribune).</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
@@ -10391,7 +10398,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Mon Oct 19</t>
+          <t>Wed Oct 14</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -10401,7 +10408,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Post Social Post 3 (details) and a Story. Email or text your personal list with a personal invite.</t>
+          <t>Post Social Post 4 (guide).</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
@@ -10409,7 +10416,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Oct 19 to 23</t>
+          <t>Mon Oct 19</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -10419,7 +10426,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Second pass: Priority B places near Proctor and 6th Ave. Return to anyone who asked you to come back.</t>
+          <t>Post Social Post 3 (details) and a Story. Email or text your personal list with a personal invite.</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
@@ -10427,17 +10434,17 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Thu Oct 22</t>
+          <t>Oct 19 to 23</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Camella and team</t>
+          <t>Camella</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>DECISION POINT: compare registrations to the goal. If well behind, widen outreach (Priority B/C, personal invites) and ask partners for a newsletter mention.</t>
+          <t>Second pass: Priority B places near Proctor and 6th Ave. Return to anyone who asked you to come back.</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr"/>
@@ -10445,17 +10452,17 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Mon Oct 26</t>
+          <t>Thu Oct 22</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Camella</t>
+          <t>Camella and team</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Early bird countdown: Story 2 and a Facebook page post ("Early bird ends Thursday").</t>
+          <t>DECISION POINT: compare registrations to the goal. If well behind, widen outreach (Priority B/C, personal invites) and ask partners for a newsletter mention.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr"/>
@@ -10463,7 +10470,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Thu Oct 29</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -10473,7 +10480,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Last day of $35 early bird. Reminder post in the morning.</t>
+          <t>Early bird countdown: Story 2 and a Facebook page post ("Early bird ends Thursday").</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
@@ -10481,7 +10488,7 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Mon Nov 2</t>
+          <t>Thu Oct 29</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -10491,7 +10498,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Post Social Post 4 (guides). Send reminder to everyone registered (time, address, parking, what to bring).</t>
+          <t>Last day of $35 early bird for both Thursdays. Reminder post in the morning.</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
@@ -10499,7 +10506,7 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Wed Nov 4</t>
+          <t>Mon Nov 2</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -10509,7 +10516,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Day-before reminder on the page and Facebook Event. Confirm venue access, refreshments and printed survey.</t>
+          <t>Text post that Nov 5 is this week and Nov 12 is next (no graphic). Send reminder to everyone registered for Nov 5 (time, address, parking, what to bring).</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
@@ -10517,17 +10524,17 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Thu Nov 5</t>
+          <t>Wed Nov 4</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>All three guides</t>
+          <t>Camella</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>EVENT. Resource table with partner brochures. Hand out the short feedback survey at the end.</t>
+          <t>Day-before reminder on the page and the Nov 5 Facebook Event. Confirm Boardroom access, refreshments and printed survey.</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr"/>
@@ -10535,25 +10542,115 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
+          <t>Thu Nov 5</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>One of the three guides</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>FIRST SESSION. Resource table with partner brochures. Hand out the short feedback survey at the end.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
           <t>Fri Nov 6</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Camella</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Thank-you message, survey summary, announce the next session to everyone who attended.</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr"/>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Thank-you message to the Nov 5 group and survey summary. Offer Nov 12 to anyone who still wants to join.</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Mon Nov 9</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Camella</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Text post that Nov 12 is this week (no graphic). Send reminder to everyone registered for Nov 12 (time, address, parking, what to bring).</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Wed Nov 11</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Camella</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Day-before reminder on the page and the Nov 12 Facebook Event. Confirm Boardroom access, refreshments and printed survey.</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Thu Nov 12</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>One of the three guides</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>SECOND SESSION. Resource table with partner brochures. Hand out the short feedback survey at the end.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Fri Nov 13</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Camella</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Thank-you message, survey summary of both sessions, announce the next session to everyone who attended.</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D22"/>
+  <autoFilter ref="A1:D27"/>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>",Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>